<commit_message>
Initial implementation of taper as design variable. Needs code cleanup but seems to work reasonably?
</commit_message>
<xml_diff>
--- a/Validation/X22 ducted propeller design.xlsx
+++ b/Validation/X22 ducted propeller design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b266c95a83fbf4bb/Documenten/TU Delft Aerospace Engineering/Msc2/AE5222 - Thesis/Software/Conceptual-Investigation-of-Alternative-Electric-Ducted-Fan-Architectures/Validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/thomasvermeule_tudelft_nl/Documents/Documents/UDC and Optimisation Framework/AircraftDuctedFanOptimisation/Validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{85ED6776-C4D8-4E62-AB2A-AD3DD39C3C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F19FF47B-95FF-466B-AAB6-86FD57B766AC}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{85ED6776-C4D8-4E62-AB2A-AD3DD39C3C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4800C198-1420-4792-8681-FD53BF422F4A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{09A38DA9-5803-4F4A-AC50-1ACCD92E16A7}"/>
+    <workbookView xWindow="-38510" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{09A38DA9-5803-4F4A-AC50-1ACCD92E16A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>r/R</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>c</t>
+  </si>
+  <si>
+    <t>taper</t>
   </si>
 </sst>
 </file>
@@ -1000,6 +1003,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1007,7 +1011,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1818,6 +1821,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1825,7 +1829,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:blipFill dpi="0" rotWithShape="1">
@@ -3373,14 +3376,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7245FA60-43DF-4342-887B-332FC6F471CF}">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3411,13 +3414,16 @@
       <c r="M1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0.2</v>
       </c>
       <c r="B2">
-        <f>A2*$G$2/2</f>
+        <f t="shared" ref="B2:B18" si="0">A2*$G$2/2</f>
         <v>0.21335999999999999</v>
       </c>
       <c r="C2">
@@ -3451,24 +3457,28 @@
         <f>D2</f>
         <v>62.6</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O2">
+        <f>L2/L2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>0.25</v>
       </c>
       <c r="B3">
-        <f>A3*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.26669999999999999</v>
       </c>
       <c r="C3">
         <v>50</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D18" si="0">$G$4+(C3-$C$13)</f>
+        <f t="shared" ref="D3:D18" si="1">$G$4+(C3-$C$13)</f>
         <v>59</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E18" si="1">$H$4+(C3-$C$18)</f>
+        <f t="shared" ref="E3:E18" si="2">$H$4+(C3-$C$18)</f>
         <v>49</v>
       </c>
       <c r="F3">
@@ -3481,35 +3491,39 @@
         <v>24</v>
       </c>
       <c r="K3">
-        <f t="shared" ref="K3:K18" si="2">B3</f>
+        <f t="shared" ref="K3:K18" si="3">B3</f>
         <v>0.26669999999999999</v>
       </c>
       <c r="L3">
-        <f t="shared" ref="L3:L18" si="3">F3</f>
+        <f t="shared" ref="L3:L18" si="4">F3</f>
         <v>0.33019999999999999</v>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M18" si="4">D3</f>
+        <f t="shared" ref="M3:M18" si="5">D3</f>
         <v>59</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O3">
+        <f>L3/L2</f>
+        <v>0.94074074074074077</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.3</v>
       </c>
       <c r="B4">
-        <f>A4*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.32003999999999999</v>
       </c>
       <c r="C4">
         <v>46.8</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>55.8</v>
       </c>
       <c r="E4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>45.8</v>
       </c>
       <c r="F4">
@@ -3522,35 +3536,39 @@
         <v>14.5</v>
       </c>
       <c r="K4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.32003999999999999</v>
       </c>
       <c r="L4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.31519999999999998</v>
       </c>
       <c r="M4">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>55.8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O4">
+        <f t="shared" ref="O4:O18" si="6">L4/L3</f>
+        <v>0.95457298606904906</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>0.35</v>
       </c>
       <c r="B5">
-        <f>A5*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.37337999999999999</v>
       </c>
       <c r="C5">
         <v>43.2</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>52.2</v>
       </c>
       <c r="E5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>42.2</v>
       </c>
       <c r="F5">
@@ -3560,35 +3578,39 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.37337999999999999</v>
       </c>
       <c r="L5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.29559999999999997</v>
       </c>
       <c r="M5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>52.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O5">
+        <f t="shared" si="6"/>
+        <v>0.93781725888324874</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>0.4</v>
       </c>
       <c r="B6">
-        <f>A6*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.42671999999999999</v>
       </c>
       <c r="C6">
         <v>39.5</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>48.5</v>
       </c>
       <c r="E6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>38.5</v>
       </c>
       <c r="F6">
@@ -3599,70 +3621,78 @@
         <v>1.2445999999999999</v>
       </c>
       <c r="K6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.42671999999999999</v>
       </c>
       <c r="L6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.27939999999999998</v>
       </c>
       <c r="M6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>48.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O6">
+        <f t="shared" si="6"/>
+        <v>0.94519621109607577</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>0.45</v>
       </c>
       <c r="B7">
-        <f>A7*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.48005999999999999</v>
       </c>
       <c r="C7">
         <v>35.9</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>44.9</v>
       </c>
       <c r="E7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>34.9</v>
       </c>
       <c r="F7">
         <v>0.26440000000000002</v>
       </c>
       <c r="K7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.48005999999999999</v>
       </c>
       <c r="L7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.26440000000000002</v>
       </c>
       <c r="M7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>44.9</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O7">
+        <f t="shared" si="6"/>
+        <v>0.94631352899069454</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>0.5</v>
       </c>
       <c r="B8">
-        <f>A8*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.53339999999999999</v>
       </c>
       <c r="C8">
         <v>32.299999999999997</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>41.3</v>
       </c>
       <c r="E8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>31.299999999999997</v>
       </c>
       <c r="F8">
@@ -3672,35 +3702,39 @@
         <v>7</v>
       </c>
       <c r="K8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.53339999999999999</v>
       </c>
       <c r="L8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.25280000000000002</v>
       </c>
       <c r="M8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>41.3</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O8">
+        <f t="shared" si="6"/>
+        <v>0.95612708018154313</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>0.55000000000000004</v>
       </c>
       <c r="B9">
-        <f>A9*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.58674000000000004</v>
       </c>
       <c r="C9">
         <v>29.1</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>38.1</v>
       </c>
       <c r="E9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>28.1</v>
       </c>
       <c r="F9">
@@ -3711,70 +3745,78 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="K9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.58674000000000004</v>
       </c>
       <c r="L9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.24479999999999999</v>
       </c>
       <c r="M9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>38.1</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O9">
+        <f t="shared" si="6"/>
+        <v>0.96835443037974667</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>0.6</v>
       </c>
       <c r="B10">
-        <f>A10*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.64007999999999998</v>
       </c>
       <c r="C10">
         <v>26.4</v>
       </c>
       <c r="D10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>35.4</v>
       </c>
       <c r="E10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>25.4</v>
       </c>
       <c r="F10">
         <v>0.24129999999999999</v>
       </c>
       <c r="K10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.64007999999999998</v>
       </c>
       <c r="L10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.24129999999999999</v>
       </c>
       <c r="M10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>35.4</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O10">
+        <f t="shared" si="6"/>
+        <v>0.98570261437908491</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>0.65</v>
       </c>
       <c r="B11">
-        <f>A11*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.69342000000000004</v>
       </c>
       <c r="C11">
         <v>24.1</v>
       </c>
       <c r="D11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>33.1</v>
       </c>
       <c r="E11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>23.1</v>
       </c>
       <c r="F11">
@@ -3784,35 +3826,39 @@
         <v>10</v>
       </c>
       <c r="K11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.69342000000000004</v>
       </c>
       <c r="L11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.23899999999999999</v>
       </c>
       <c r="M11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>33.1</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O11">
+        <f t="shared" si="6"/>
+        <v>0.99046829672606718</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>0.7</v>
       </c>
       <c r="B12">
-        <f>A12*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.74675999999999998</v>
       </c>
       <c r="C12">
         <v>21.8</v>
       </c>
       <c r="D12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>30.8</v>
       </c>
       <c r="E12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20.8</v>
       </c>
       <c r="F12">
@@ -3823,226 +3869,254 @@
         <v>0.35560000000000003</v>
       </c>
       <c r="K12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.74675999999999998</v>
       </c>
       <c r="L12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.23669999999999999</v>
       </c>
       <c r="M12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>30.8</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O12">
+        <f t="shared" si="6"/>
+        <v>0.99037656903765692</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>0.75</v>
       </c>
       <c r="B13">
-        <f>A13*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.80010000000000003</v>
       </c>
       <c r="C13">
         <v>20</v>
       </c>
       <c r="D13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="E13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="F13">
         <v>0.23319999999999999</v>
       </c>
       <c r="K13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.80010000000000003</v>
       </c>
       <c r="L13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.23319999999999999</v>
       </c>
       <c r="M13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O13">
+        <f t="shared" si="6"/>
+        <v>0.98521335023236167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>0.8</v>
       </c>
       <c r="B14">
-        <f>A14*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.85343999999999998</v>
       </c>
       <c r="C14">
         <v>19.100000000000001</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28.1</v>
       </c>
       <c r="E14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18.100000000000001</v>
       </c>
       <c r="F14">
         <v>0.23089999999999999</v>
       </c>
       <c r="K14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.85343999999999998</v>
       </c>
       <c r="L14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.23089999999999999</v>
       </c>
       <c r="M14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>28.1</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O14">
+        <f t="shared" si="6"/>
+        <v>0.99013722126929671</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>0.85</v>
       </c>
       <c r="B15">
-        <f>A15*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.90677999999999992</v>
       </c>
       <c r="C15">
         <v>17.7</v>
       </c>
       <c r="D15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26.7</v>
       </c>
       <c r="E15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16.7</v>
       </c>
       <c r="F15">
         <v>0.2286</v>
       </c>
       <c r="K15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.90677999999999992</v>
       </c>
       <c r="L15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.2286</v>
       </c>
       <c r="M15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>26.7</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O15">
+        <f t="shared" si="6"/>
+        <v>0.99003897791251627</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>0.9</v>
       </c>
       <c r="B16">
-        <f>A16*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>0.96011999999999997</v>
       </c>
       <c r="C16">
         <v>16.8</v>
       </c>
       <c r="D16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>25.8</v>
       </c>
       <c r="E16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15.8</v>
       </c>
       <c r="F16">
         <v>0.22509999999999999</v>
       </c>
       <c r="K16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.96011999999999997</v>
       </c>
       <c r="L16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.22509999999999999</v>
       </c>
       <c r="M16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>25.8</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O16">
+        <f t="shared" si="6"/>
+        <v>0.98468941382327213</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>0.95</v>
       </c>
       <c r="B17">
-        <f>A17*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>1.01346</v>
       </c>
       <c r="C17">
         <v>15.9</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24.9</v>
       </c>
       <c r="E17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.9</v>
       </c>
       <c r="F17">
         <v>0.22170000000000001</v>
       </c>
       <c r="K17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.01346</v>
       </c>
       <c r="L17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.22170000000000001</v>
       </c>
       <c r="M17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>24.9</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="O17">
+        <f t="shared" si="6"/>
+        <v>0.98489560195468684</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1</v>
       </c>
       <c r="B18">
-        <f>A18*$G$2/2</f>
+        <f t="shared" si="0"/>
         <v>1.0668</v>
       </c>
       <c r="C18">
         <v>15.5</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24.5</v>
       </c>
       <c r="E18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.5</v>
       </c>
       <c r="F18">
         <v>0.2205</v>
       </c>
       <c r="K18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0668</v>
       </c>
       <c r="L18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.2205</v>
       </c>
       <c r="M18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>24.5</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="6"/>
+        <v>0.99458728010825437</v>
       </c>
     </row>
   </sheetData>

</xml_diff>